<commit_message>
results from test with updates to the data formatting and upload module
</commit_message>
<xml_diff>
--- a/results/02_post_QA_QC_transcribed_hydroclimate_data/508/508_198802_SF.JPG_post_QA_QC.xlsx
+++ b/results/02_post_QA_QC_transcribed_hydroclimate_data/508/508_198802_SF.JPG_post_QA_QC.xlsx
@@ -820,13 +820,13 @@
       <c r="M4" s="11" t="n">
         <v>18.4</v>
       </c>
-      <c r="N4" s="3" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="P4" s="3" t="n">
+      <c r="N4" s="11" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="O4" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="P4" s="11" t="n">
         <v>0</v>
       </c>
       <c r="Q4" s="11" t="n">
@@ -899,13 +899,13 @@
       <c r="M5" s="11" t="n">
         <v>17.6</v>
       </c>
-      <c r="N5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O5" s="3" t="n">
-        <v>91.2</v>
-      </c>
-      <c r="P5" s="3" t="n">
+      <c r="N5" s="11" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="O5" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="P5" s="11" t="n">
         <v>0</v>
       </c>
       <c r="Q5" s="11" t="n">
@@ -982,14 +982,14 @@
       <c r="M6" s="11" t="n">
         <v>17.5</v>
       </c>
-      <c r="N6" s="3" t="n">
-        <v>15.8</v>
-      </c>
-      <c r="O6" s="3" t="n">
-        <v>91.2</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>2</v>
+      <c r="N6" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="O6" s="11" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="P6" s="11" t="n">
+        <v>-0.1</v>
       </c>
       <c r="Q6" s="11" t="n">
         <v>29.5</v>
@@ -1065,26 +1065,28 @@
       <c r="M7" s="11" t="n">
         <v>20.4</v>
       </c>
-      <c r="N7" s="3" t="inlineStr"/>
-      <c r="O7" s="3" t="n">
-        <v>90.59999999999999</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>0.2</v>
+      <c r="N7" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="O7" s="11" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="P7" s="11" t="n">
+        <v>-0.1</v>
       </c>
       <c r="Q7" s="11" t="n">
         <v>20.1</v>
       </c>
-      <c r="R7" s="3" t="n">
+      <c r="R7" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="S7" s="3" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="T7" s="3" t="n">
-        <v>87.2</v>
-      </c>
-      <c r="U7" s="3" t="n">
+      <c r="S7" s="11" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="T7" s="11" t="n">
+        <v>96.2</v>
+      </c>
+      <c r="U7" s="11" t="n">
         <v>0.9</v>
       </c>
       <c r="V7" s="3" t="n">
@@ -1148,12 +1150,14 @@
       <c r="M8" s="11" t="n">
         <v>18.9</v>
       </c>
-      <c r="N8" s="3" t="inlineStr"/>
-      <c r="O8" s="3" t="n">
-        <v>91.2</v>
-      </c>
-      <c r="P8" s="3" t="n">
-        <v>8</v>
+      <c r="N8" s="11" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="O8" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="P8" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="Q8" s="11" t="n">
         <v>25.8</v>
@@ -1312,14 +1316,14 @@
       <c r="M10" s="11" t="n">
         <v>18.5</v>
       </c>
-      <c r="N10" s="3" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="O10" s="3" t="n">
-        <v>91.2</v>
-      </c>
-      <c r="P10" s="3" t="n">
-        <v>0.1</v>
+      <c r="N10" s="11" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="O10" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="P10" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="Q10" s="11" t="n">
         <v>25.9</v>
@@ -2042,14 +2046,16 @@
       <c r="L19" s="11" t="n">
         <v>18.3</v>
       </c>
-      <c r="M19" s="3" t="n">
+      <c r="M19" s="11" t="n">
         <v>18.2</v>
       </c>
-      <c r="N19" s="3" t="inlineStr"/>
-      <c r="O19" s="3" t="n">
-        <v>92.2</v>
-      </c>
-      <c r="P19" s="3" t="n">
+      <c r="N19" s="11" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="O19" s="11" t="n">
+        <v>99</v>
+      </c>
+      <c r="P19" s="11" t="n">
         <v>0.2</v>
       </c>
       <c r="Q19" s="3" t="n">
@@ -2121,16 +2127,16 @@
       <c r="L20" s="11" t="n">
         <v>19.2</v>
       </c>
-      <c r="M20" s="3" t="n">
+      <c r="M20" s="11" t="n">
         <v>19.2</v>
       </c>
-      <c r="N20" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="O20" s="3" t="n">
-        <v>90.2</v>
-      </c>
-      <c r="P20" s="3" t="n">
+      <c r="N20" s="11" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="O20" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="P20" s="11" t="n">
         <v>0</v>
       </c>
       <c r="Q20" s="15" t="n">
@@ -2279,16 +2285,16 @@
       <c r="L22" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="M22" s="3" t="n">
+      <c r="M22" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="N22" s="3" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="O22" s="3" t="n">
-        <v>99.2</v>
-      </c>
-      <c r="P22" s="3" t="n">
+      <c r="N22" s="11" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="O22" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="P22" s="11" t="n">
         <v>0</v>
       </c>
       <c r="Q22" s="3" t="n">
@@ -3085,14 +3091,14 @@
       <c r="R32" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="S32" s="3" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="T32" s="3" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="U32" s="3" t="n">
-        <v>15.5</v>
+      <c r="S32" s="11" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="T32" s="11" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="U32" s="11" t="n">
+        <v>12.4</v>
       </c>
       <c r="V32" s="3" t="n">
         <v>22.2</v>
@@ -3162,14 +3168,14 @@
       <c r="R33" s="11" t="n">
         <v>27.8</v>
       </c>
-      <c r="S33" s="3" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="T33" s="3" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="U33" s="3" t="n">
-        <v>15</v>
+      <c r="S33" s="11" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="T33" s="11" t="n">
+        <v>93.8</v>
+      </c>
+      <c r="U33" s="11" t="n">
+        <v>2.5</v>
       </c>
       <c r="V33" s="3" t="n">
         <v>29.2</v>
@@ -3243,14 +3249,14 @@
       <c r="R34" s="11" t="n">
         <v>20.9</v>
       </c>
-      <c r="S34" s="3" t="n">
-        <v>22.3</v>
-      </c>
-      <c r="T34" s="3" t="n">
-        <v>69.2</v>
-      </c>
-      <c r="U34" s="3" t="n">
-        <v>2</v>
+      <c r="S34" s="11" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="T34" s="11" t="n">
+        <v>78.90000000000001</v>
+      </c>
+      <c r="U34" s="11" t="n">
+        <v>6.6</v>
       </c>
       <c r="V34" s="3" t="n">
         <v>20</v>
@@ -3324,14 +3330,14 @@
       <c r="R35" s="11" t="n">
         <v>22.8</v>
       </c>
-      <c r="S35" s="3" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="T35" s="3" t="n">
-        <v>192.2</v>
-      </c>
-      <c r="U35" s="3" t="n">
-        <v>2.5</v>
+      <c r="S35" s="11" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="T35" s="11" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="U35" s="11" t="n">
+        <v>10.1</v>
       </c>
       <c r="V35" s="3" t="n">
         <v>32</v>
@@ -3403,14 +3409,14 @@
       <c r="R36" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="S36" s="3" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="T36" s="3" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="U36" s="3" t="n">
-        <v>2.8</v>
+      <c r="S36" s="11" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="T36" s="11" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="U36" s="11" t="n">
+        <v>17.4</v>
       </c>
       <c r="V36" s="3" t="n">
         <v>23.9</v>
@@ -3563,14 +3569,14 @@
       <c r="R38" s="11" t="n">
         <v>23.5</v>
       </c>
-      <c r="S38" s="3" t="n">
-        <v>28.1</v>
-      </c>
-      <c r="T38" s="3" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="U38" s="3" t="n">
-        <v>24.9</v>
+      <c r="S38" s="11" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="T38" s="11" t="n">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="U38" s="11" t="n">
+        <v>10.2</v>
       </c>
       <c r="V38" s="9" t="n">
         <v>22.2</v>

</xml_diff>